<commit_message>
Faculty Login Logic Change/
</commit_message>
<xml_diff>
--- a/backend/DATA_SYSTEM.xlsx
+++ b/backend/DATA_SYSTEM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Randel\Downloads\Von Files\Von_Thesis\Von_Thesis\venv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Randel\Downloads\Von Files\Von_Thesis\Von_Thesis\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DF56B6-D0A1-4FCB-BEF1-7F43332F63EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC874D0-E5EE-4372-82CE-1C1CA4330EEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25673,7 +25673,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H334"/>
+  <dimension ref="A1:H251"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.42578125" customWidth="1"/>
@@ -32368,836 +32368,6 @@
       <c r="H251" s="25">
         <v>45505</v>
       </c>
-    </row>
-    <row r="252" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A252" s="18"/>
-      <c r="B252" s="12"/>
-      <c r="C252" s="12"/>
-      <c r="D252" s="12"/>
-      <c r="E252" s="7"/>
-      <c r="F252" s="8"/>
-      <c r="G252" s="22"/>
-      <c r="H252" s="25"/>
-    </row>
-    <row r="253" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A253" s="11"/>
-      <c r="B253" s="12"/>
-      <c r="C253" s="12"/>
-      <c r="D253" s="12"/>
-      <c r="E253" s="7"/>
-      <c r="F253" s="8"/>
-      <c r="G253" s="22"/>
-      <c r="H253" s="25"/>
-    </row>
-    <row r="254" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A254" s="11"/>
-      <c r="B254" s="12"/>
-      <c r="C254" s="12"/>
-      <c r="D254" s="12"/>
-      <c r="E254" s="7"/>
-      <c r="F254" s="8"/>
-      <c r="G254" s="22"/>
-      <c r="H254" s="25"/>
-    </row>
-    <row r="255" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A255" s="11"/>
-      <c r="B255" s="12"/>
-      <c r="C255" s="12"/>
-      <c r="D255" s="12"/>
-      <c r="E255" s="7"/>
-      <c r="F255" s="8"/>
-      <c r="G255" s="22"/>
-      <c r="H255" s="25"/>
-    </row>
-    <row r="256" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A256" s="11"/>
-      <c r="B256" s="12"/>
-      <c r="C256" s="12"/>
-      <c r="D256" s="12"/>
-      <c r="E256" s="7"/>
-      <c r="F256" s="8"/>
-      <c r="G256" s="22"/>
-      <c r="H256" s="25"/>
-    </row>
-    <row r="257" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A257" s="11"/>
-      <c r="B257" s="12"/>
-      <c r="C257" s="12"/>
-      <c r="D257" s="12"/>
-      <c r="E257" s="7"/>
-      <c r="F257" s="8"/>
-      <c r="G257" s="22"/>
-      <c r="H257" s="25"/>
-    </row>
-    <row r="258" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A258" s="11"/>
-      <c r="B258" s="12"/>
-      <c r="C258" s="12"/>
-      <c r="D258" s="12"/>
-      <c r="E258" s="7"/>
-      <c r="F258" s="8"/>
-      <c r="G258" s="22"/>
-      <c r="H258" s="25"/>
-    </row>
-    <row r="259" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A259" s="11"/>
-      <c r="B259" s="12"/>
-      <c r="C259" s="12"/>
-      <c r="D259" s="12"/>
-      <c r="E259" s="7"/>
-      <c r="F259" s="8"/>
-      <c r="G259" s="22"/>
-      <c r="H259" s="25"/>
-    </row>
-    <row r="260" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A260" s="11"/>
-      <c r="B260" s="12"/>
-      <c r="C260" s="12"/>
-      <c r="D260" s="12"/>
-      <c r="E260" s="7"/>
-      <c r="F260" s="8"/>
-      <c r="G260" s="22"/>
-      <c r="H260" s="25"/>
-    </row>
-    <row r="261" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A261" s="11"/>
-      <c r="B261" s="12"/>
-      <c r="C261" s="12"/>
-      <c r="D261" s="12"/>
-      <c r="E261" s="7"/>
-      <c r="F261" s="8"/>
-      <c r="G261" s="22"/>
-      <c r="H261" s="25"/>
-    </row>
-    <row r="262" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A262" s="11"/>
-      <c r="B262" s="12"/>
-      <c r="C262" s="12"/>
-      <c r="D262" s="12"/>
-      <c r="E262" s="7"/>
-      <c r="F262" s="8"/>
-      <c r="G262" s="22"/>
-      <c r="H262" s="25"/>
-    </row>
-    <row r="263" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A263" s="11"/>
-      <c r="B263" s="12"/>
-      <c r="C263" s="12"/>
-      <c r="D263" s="12"/>
-      <c r="E263" s="7"/>
-      <c r="F263" s="8"/>
-      <c r="G263" s="22"/>
-      <c r="H263" s="25"/>
-    </row>
-    <row r="264" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A264" s="11"/>
-      <c r="B264" s="12"/>
-      <c r="C264" s="12"/>
-      <c r="D264" s="12"/>
-      <c r="E264" s="7"/>
-      <c r="F264" s="8"/>
-      <c r="G264" s="22"/>
-      <c r="H264" s="25"/>
-    </row>
-    <row r="265" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A265" s="11"/>
-      <c r="B265" s="12"/>
-      <c r="C265" s="12"/>
-      <c r="D265" s="12"/>
-      <c r="E265" s="7"/>
-      <c r="F265" s="8"/>
-      <c r="G265" s="22"/>
-      <c r="H265" s="25"/>
-    </row>
-    <row r="266" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A266" s="11"/>
-      <c r="B266" s="12"/>
-      <c r="C266" s="12"/>
-      <c r="D266" s="12"/>
-      <c r="E266" s="7"/>
-      <c r="F266" s="8"/>
-      <c r="G266" s="22"/>
-      <c r="H266" s="25"/>
-    </row>
-    <row r="267" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A267" s="11"/>
-      <c r="B267" s="12"/>
-      <c r="C267" s="12"/>
-      <c r="D267" s="12"/>
-      <c r="E267" s="7"/>
-      <c r="F267" s="8"/>
-      <c r="G267" s="22"/>
-      <c r="H267" s="25"/>
-    </row>
-    <row r="268" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A268" s="11"/>
-      <c r="B268" s="12"/>
-      <c r="C268" s="12"/>
-      <c r="D268" s="12"/>
-      <c r="E268" s="7"/>
-      <c r="F268" s="8"/>
-      <c r="G268" s="22"/>
-      <c r="H268" s="25"/>
-    </row>
-    <row r="269" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A269" s="11"/>
-      <c r="B269" s="12"/>
-      <c r="C269" s="12"/>
-      <c r="D269" s="12"/>
-      <c r="E269" s="7"/>
-      <c r="F269" s="8"/>
-      <c r="G269" s="20"/>
-      <c r="H269" s="25"/>
-    </row>
-    <row r="270" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A270" s="11"/>
-      <c r="B270" s="12"/>
-      <c r="C270" s="12"/>
-      <c r="D270" s="12"/>
-      <c r="E270" s="7"/>
-      <c r="F270" s="8"/>
-      <c r="G270" s="22"/>
-      <c r="H270" s="25"/>
-    </row>
-    <row r="271" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A271" s="11"/>
-      <c r="B271" s="12"/>
-      <c r="C271" s="12"/>
-      <c r="D271" s="12"/>
-      <c r="E271" s="7"/>
-      <c r="F271" s="8"/>
-      <c r="G271" s="22"/>
-      <c r="H271" s="25"/>
-    </row>
-    <row r="272" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A272" s="11"/>
-      <c r="B272" s="12"/>
-      <c r="C272" s="12"/>
-      <c r="D272" s="12"/>
-      <c r="E272" s="7"/>
-      <c r="F272" s="8"/>
-      <c r="G272" s="22"/>
-      <c r="H272" s="25"/>
-    </row>
-    <row r="273" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A273" s="11"/>
-      <c r="B273" s="12"/>
-      <c r="C273" s="12"/>
-      <c r="D273" s="12"/>
-      <c r="E273" s="7"/>
-      <c r="F273" s="8"/>
-      <c r="G273" s="22"/>
-      <c r="H273" s="25"/>
-    </row>
-    <row r="274" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A274" s="11"/>
-      <c r="B274" s="12"/>
-      <c r="C274" s="12"/>
-      <c r="D274" s="12"/>
-      <c r="E274" s="7"/>
-      <c r="F274" s="8"/>
-      <c r="G274" s="23"/>
-      <c r="H274" s="26"/>
-    </row>
-    <row r="275" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A275" s="11"/>
-      <c r="B275" s="12"/>
-      <c r="C275" s="12"/>
-      <c r="D275" s="12"/>
-      <c r="E275" s="7"/>
-      <c r="F275" s="8"/>
-      <c r="G275" s="23"/>
-      <c r="H275" s="26"/>
-    </row>
-    <row r="276" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A276" s="11"/>
-      <c r="B276" s="12"/>
-      <c r="C276" s="12"/>
-      <c r="D276" s="12"/>
-      <c r="E276" s="7"/>
-      <c r="F276" s="8"/>
-      <c r="G276" s="23"/>
-      <c r="H276" s="26"/>
-    </row>
-    <row r="277" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A277" s="11"/>
-      <c r="B277" s="12"/>
-      <c r="C277" s="12"/>
-      <c r="D277" s="12"/>
-      <c r="E277" s="7"/>
-      <c r="F277" s="8"/>
-      <c r="G277" s="23"/>
-      <c r="H277" s="26"/>
-    </row>
-    <row r="278" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A278" s="11"/>
-      <c r="B278" s="12"/>
-      <c r="C278" s="12"/>
-      <c r="D278" s="12"/>
-      <c r="E278" s="7"/>
-      <c r="F278" s="8"/>
-      <c r="G278" s="23"/>
-      <c r="H278" s="26"/>
-    </row>
-    <row r="279" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A279" s="11"/>
-      <c r="B279" s="12"/>
-      <c r="C279" s="12"/>
-      <c r="D279" s="12"/>
-      <c r="E279" s="7"/>
-      <c r="F279" s="8"/>
-      <c r="G279" s="23"/>
-      <c r="H279" s="26"/>
-    </row>
-    <row r="280" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A280" s="11"/>
-      <c r="B280" s="12"/>
-      <c r="C280" s="12"/>
-      <c r="D280" s="12"/>
-      <c r="E280" s="7"/>
-      <c r="F280" s="8"/>
-      <c r="G280" s="23"/>
-      <c r="H280" s="26"/>
-    </row>
-    <row r="281" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A281" s="11"/>
-      <c r="B281" s="12"/>
-      <c r="C281" s="12"/>
-      <c r="D281" s="12"/>
-      <c r="E281" s="7"/>
-      <c r="F281" s="8"/>
-      <c r="G281" s="22"/>
-      <c r="H281" s="25"/>
-    </row>
-    <row r="282" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A282" s="11"/>
-      <c r="B282" s="12"/>
-      <c r="C282" s="12"/>
-      <c r="D282" s="12"/>
-      <c r="E282" s="7"/>
-      <c r="F282" s="8"/>
-      <c r="G282" s="22"/>
-      <c r="H282" s="25"/>
-    </row>
-    <row r="283" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A283" s="11"/>
-      <c r="B283" s="12"/>
-      <c r="C283" s="12"/>
-      <c r="D283" s="12"/>
-      <c r="E283" s="7"/>
-      <c r="F283" s="8"/>
-      <c r="G283" s="22"/>
-      <c r="H283" s="25"/>
-    </row>
-    <row r="284" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A284" s="11"/>
-      <c r="B284" s="12"/>
-      <c r="C284" s="12"/>
-      <c r="D284" s="12"/>
-      <c r="E284" s="7"/>
-      <c r="F284" s="8"/>
-      <c r="G284" s="22"/>
-      <c r="H284" s="25"/>
-    </row>
-    <row r="285" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A285" s="11"/>
-      <c r="B285" s="12"/>
-      <c r="C285" s="12"/>
-      <c r="D285" s="12"/>
-      <c r="E285" s="7"/>
-      <c r="F285" s="8"/>
-      <c r="G285" s="20"/>
-      <c r="H285" s="25"/>
-    </row>
-    <row r="286" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A286" s="11"/>
-      <c r="B286" s="12"/>
-      <c r="C286" s="12"/>
-      <c r="D286" s="12"/>
-      <c r="E286" s="7"/>
-      <c r="F286" s="8"/>
-      <c r="G286" s="22"/>
-      <c r="H286" s="25"/>
-    </row>
-    <row r="287" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A287" s="11"/>
-      <c r="B287" s="12"/>
-      <c r="C287" s="12"/>
-      <c r="D287" s="12"/>
-      <c r="E287" s="7"/>
-      <c r="F287" s="8"/>
-      <c r="G287" s="22"/>
-      <c r="H287" s="25"/>
-    </row>
-    <row r="288" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A288" s="11"/>
-      <c r="B288" s="12"/>
-      <c r="C288" s="12"/>
-      <c r="D288" s="12"/>
-      <c r="E288" s="7"/>
-      <c r="F288" s="8"/>
-      <c r="G288" s="22"/>
-      <c r="H288" s="25"/>
-    </row>
-    <row r="289" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A289" s="11"/>
-      <c r="B289" s="12"/>
-      <c r="C289" s="12"/>
-      <c r="D289" s="12"/>
-      <c r="E289" s="10"/>
-      <c r="F289" s="8"/>
-      <c r="G289" s="20"/>
-      <c r="H289" s="25"/>
-    </row>
-    <row r="290" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A290" s="11"/>
-      <c r="B290" s="12"/>
-      <c r="C290" s="12"/>
-      <c r="D290" s="12"/>
-      <c r="E290" s="10"/>
-      <c r="F290" s="8"/>
-      <c r="G290" s="22"/>
-      <c r="H290" s="25"/>
-    </row>
-    <row r="291" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A291" s="11"/>
-      <c r="B291" s="12"/>
-      <c r="C291" s="12"/>
-      <c r="D291" s="12"/>
-      <c r="E291" s="10"/>
-      <c r="F291" s="8"/>
-      <c r="G291" s="22"/>
-      <c r="H291" s="25"/>
-    </row>
-    <row r="292" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A292" s="11"/>
-      <c r="B292" s="12"/>
-      <c r="C292" s="12"/>
-      <c r="D292" s="12"/>
-      <c r="E292" s="10"/>
-      <c r="F292" s="8"/>
-      <c r="G292" s="22"/>
-      <c r="H292" s="25"/>
-    </row>
-    <row r="293" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A293" s="11"/>
-      <c r="B293" s="12"/>
-      <c r="C293" s="12"/>
-      <c r="D293" s="12"/>
-      <c r="E293" s="10"/>
-      <c r="F293" s="8"/>
-      <c r="G293" s="22"/>
-      <c r="H293" s="25"/>
-    </row>
-    <row r="294" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A294" s="11"/>
-      <c r="B294" s="12"/>
-      <c r="C294" s="12"/>
-      <c r="D294" s="12"/>
-      <c r="E294" s="10"/>
-      <c r="F294" s="8"/>
-      <c r="G294" s="22"/>
-      <c r="H294" s="25"/>
-    </row>
-    <row r="295" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A295" s="11"/>
-      <c r="B295" s="12"/>
-      <c r="C295" s="12"/>
-      <c r="D295" s="12"/>
-      <c r="E295" s="10"/>
-      <c r="F295" s="8"/>
-      <c r="G295" s="20"/>
-      <c r="H295" s="25"/>
-    </row>
-    <row r="296" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A296" s="11"/>
-      <c r="B296" s="12"/>
-      <c r="C296" s="12"/>
-      <c r="D296" s="12"/>
-      <c r="E296" s="10"/>
-      <c r="F296" s="8"/>
-      <c r="G296" s="22"/>
-      <c r="H296" s="25"/>
-    </row>
-    <row r="297" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A297" s="11"/>
-      <c r="B297" s="12"/>
-      <c r="C297" s="12"/>
-      <c r="D297" s="12"/>
-      <c r="E297" s="10"/>
-      <c r="F297" s="8"/>
-      <c r="G297" s="23"/>
-      <c r="H297" s="26"/>
-    </row>
-    <row r="298" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A298" s="11"/>
-      <c r="B298" s="12"/>
-      <c r="C298" s="12"/>
-      <c r="D298" s="12"/>
-      <c r="E298" s="10"/>
-      <c r="F298" s="8"/>
-      <c r="G298" s="8"/>
-      <c r="H298" s="26"/>
-    </row>
-    <row r="299" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A299" s="8"/>
-      <c r="B299" s="12"/>
-      <c r="C299" s="12"/>
-      <c r="D299" s="12"/>
-      <c r="E299" s="10"/>
-      <c r="F299" s="8"/>
-      <c r="G299" s="8"/>
-      <c r="H299" s="26"/>
-    </row>
-    <row r="300" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A300" s="11"/>
-      <c r="B300" s="12"/>
-      <c r="C300" s="12"/>
-      <c r="D300" s="12"/>
-      <c r="E300" s="10"/>
-      <c r="F300" s="8"/>
-      <c r="G300" s="23"/>
-      <c r="H300" s="26"/>
-    </row>
-    <row r="301" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A301" s="11"/>
-      <c r="B301" s="12"/>
-      <c r="C301" s="12"/>
-      <c r="D301" s="12"/>
-      <c r="E301" s="10"/>
-      <c r="F301" s="8"/>
-      <c r="G301" s="23"/>
-      <c r="H301" s="26"/>
-    </row>
-    <row r="302" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A302" s="11"/>
-      <c r="B302" s="12"/>
-      <c r="C302" s="12"/>
-      <c r="D302" s="12"/>
-      <c r="E302" s="10"/>
-      <c r="F302" s="8"/>
-      <c r="G302" s="23"/>
-      <c r="H302" s="26"/>
-    </row>
-    <row r="303" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A303" s="11"/>
-      <c r="B303" s="12"/>
-      <c r="C303" s="12"/>
-      <c r="D303" s="12"/>
-      <c r="E303" s="10"/>
-      <c r="F303" s="8"/>
-      <c r="G303" s="23"/>
-      <c r="H303" s="26"/>
-    </row>
-    <row r="304" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A304" s="11"/>
-      <c r="B304" s="12"/>
-      <c r="C304" s="12"/>
-      <c r="D304" s="12"/>
-      <c r="E304" s="10"/>
-      <c r="F304" s="8"/>
-      <c r="G304" s="23"/>
-      <c r="H304" s="26"/>
-    </row>
-    <row r="305" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A305" s="11"/>
-      <c r="B305" s="12"/>
-      <c r="C305" s="12"/>
-      <c r="D305" s="12"/>
-      <c r="E305" s="10"/>
-      <c r="F305" s="8"/>
-      <c r="G305" s="8"/>
-      <c r="H305" s="26"/>
-    </row>
-    <row r="306" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A306" s="11"/>
-      <c r="B306" s="12"/>
-      <c r="C306" s="12"/>
-      <c r="D306" s="12"/>
-      <c r="E306" s="10"/>
-      <c r="F306" s="8"/>
-      <c r="G306" s="23"/>
-      <c r="H306" s="26"/>
-    </row>
-    <row r="307" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A307" s="11"/>
-      <c r="B307" s="12"/>
-      <c r="C307" s="12"/>
-      <c r="D307" s="12"/>
-      <c r="E307" s="10"/>
-      <c r="F307" s="8"/>
-      <c r="G307" s="22"/>
-      <c r="H307" s="25"/>
-    </row>
-    <row r="308" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A308" s="11"/>
-      <c r="B308" s="12"/>
-      <c r="C308" s="12"/>
-      <c r="D308" s="12"/>
-      <c r="E308" s="10"/>
-      <c r="F308" s="8"/>
-      <c r="G308" s="22"/>
-      <c r="H308" s="25"/>
-    </row>
-    <row r="309" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A309" s="11"/>
-      <c r="B309" s="12"/>
-      <c r="C309" s="12"/>
-      <c r="D309" s="12"/>
-      <c r="E309" s="10"/>
-      <c r="F309" s="8"/>
-      <c r="G309" s="22"/>
-      <c r="H309" s="25"/>
-    </row>
-    <row r="310" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A310" s="11"/>
-      <c r="B310" s="12"/>
-      <c r="C310" s="12"/>
-      <c r="D310" s="12"/>
-      <c r="E310" s="10"/>
-      <c r="F310" s="8"/>
-      <c r="G310" s="22"/>
-      <c r="H310" s="25"/>
-    </row>
-    <row r="311" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A311" s="11"/>
-      <c r="B311" s="12"/>
-      <c r="C311" s="12"/>
-      <c r="D311" s="12"/>
-      <c r="E311" s="10"/>
-      <c r="F311" s="8"/>
-      <c r="G311" s="22"/>
-      <c r="H311" s="25"/>
-    </row>
-    <row r="312" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A312" s="11"/>
-      <c r="B312" s="12"/>
-      <c r="C312" s="12"/>
-      <c r="D312" s="12"/>
-      <c r="E312" s="10"/>
-      <c r="F312" s="8"/>
-      <c r="G312" s="22"/>
-      <c r="H312" s="25"/>
-    </row>
-    <row r="313" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A313" s="11"/>
-      <c r="B313" s="12"/>
-      <c r="C313" s="12"/>
-      <c r="D313" s="12"/>
-      <c r="E313" s="7"/>
-      <c r="F313" s="8"/>
-      <c r="G313" s="22"/>
-      <c r="H313" s="25"/>
-    </row>
-    <row r="314" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A314" s="11"/>
-      <c r="B314" s="12"/>
-      <c r="C314" s="12"/>
-      <c r="D314" s="12"/>
-      <c r="E314" s="10"/>
-      <c r="F314" s="8"/>
-      <c r="G314" s="22"/>
-      <c r="H314" s="25"/>
-    </row>
-    <row r="315" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A315" s="18"/>
-      <c r="B315" s="19"/>
-      <c r="C315" s="19"/>
-      <c r="D315" s="19"/>
-      <c r="E315" s="10"/>
-      <c r="F315" s="8"/>
-      <c r="G315" s="20"/>
-      <c r="H315" s="25"/>
-    </row>
-    <row r="316" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A316" s="18"/>
-      <c r="B316" s="19"/>
-      <c r="C316" s="19"/>
-      <c r="D316" s="19"/>
-      <c r="E316" s="10"/>
-      <c r="F316" s="8"/>
-      <c r="G316" s="22"/>
-      <c r="H316" s="25"/>
-    </row>
-    <row r="317" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A317" s="18"/>
-      <c r="B317" s="19"/>
-      <c r="C317" s="19"/>
-      <c r="D317" s="19"/>
-      <c r="E317" s="10"/>
-      <c r="F317" s="8"/>
-      <c r="G317" s="22"/>
-      <c r="H317" s="25"/>
-    </row>
-    <row r="318" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A318" s="18"/>
-      <c r="B318" s="19"/>
-      <c r="C318" s="19"/>
-      <c r="D318" s="19"/>
-      <c r="E318" s="10"/>
-      <c r="F318" s="8"/>
-      <c r="G318" s="22"/>
-      <c r="H318" s="25"/>
-    </row>
-    <row r="319" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A319" s="18"/>
-      <c r="B319" s="19"/>
-      <c r="C319" s="19"/>
-      <c r="D319" s="19"/>
-      <c r="E319" s="10"/>
-      <c r="F319" s="8"/>
-      <c r="G319" s="22"/>
-      <c r="H319" s="25"/>
-    </row>
-    <row r="320" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A320" s="18"/>
-      <c r="B320" s="19"/>
-      <c r="C320" s="19"/>
-      <c r="D320" s="19"/>
-      <c r="E320" s="10"/>
-      <c r="F320" s="8"/>
-      <c r="G320" s="22"/>
-      <c r="H320" s="25"/>
-    </row>
-    <row r="321" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A321" s="18"/>
-      <c r="B321" s="19"/>
-      <c r="C321" s="19"/>
-      <c r="D321" s="19"/>
-      <c r="E321" s="10"/>
-      <c r="F321" s="8"/>
-      <c r="G321" s="22"/>
-      <c r="H321" s="25"/>
-    </row>
-    <row r="322" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A322" s="18"/>
-      <c r="B322" s="19"/>
-      <c r="C322" s="19"/>
-      <c r="D322" s="19"/>
-      <c r="E322" s="10"/>
-      <c r="F322" s="8"/>
-      <c r="G322" s="20"/>
-      <c r="H322" s="25"/>
-    </row>
-    <row r="323" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A323" s="18"/>
-      <c r="B323" s="19"/>
-      <c r="C323" s="19"/>
-      <c r="D323" s="19"/>
-      <c r="E323" s="10"/>
-      <c r="F323" s="8"/>
-      <c r="G323" s="22"/>
-      <c r="H323" s="25"/>
-    </row>
-    <row r="324" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A324" s="18"/>
-      <c r="B324" s="19"/>
-      <c r="C324" s="19"/>
-      <c r="D324" s="19"/>
-      <c r="E324" s="10"/>
-      <c r="F324" s="8"/>
-      <c r="G324" s="23"/>
-      <c r="H324" s="26"/>
-    </row>
-    <row r="325" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A325" s="18"/>
-      <c r="B325" s="19"/>
-      <c r="C325" s="19"/>
-      <c r="D325" s="19"/>
-      <c r="E325" s="10"/>
-      <c r="F325" s="8"/>
-      <c r="G325" s="23"/>
-      <c r="H325" s="26"/>
-    </row>
-    <row r="326" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A326" s="18"/>
-      <c r="B326" s="19"/>
-      <c r="C326" s="19"/>
-      <c r="D326" s="19"/>
-      <c r="E326" s="10"/>
-      <c r="F326" s="8"/>
-      <c r="G326" s="23"/>
-      <c r="H326" s="26"/>
-    </row>
-    <row r="327" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A327" s="18"/>
-      <c r="B327" s="19"/>
-      <c r="C327" s="19"/>
-      <c r="D327" s="19"/>
-      <c r="E327" s="10"/>
-      <c r="F327" s="8"/>
-      <c r="G327" s="8"/>
-      <c r="H327" s="26"/>
-    </row>
-    <row r="328" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A328" s="11"/>
-      <c r="B328" s="12"/>
-      <c r="C328" s="12"/>
-      <c r="D328" s="12"/>
-      <c r="E328" s="10"/>
-      <c r="F328" s="8"/>
-      <c r="G328" s="8"/>
-      <c r="H328" s="26"/>
-    </row>
-    <row r="329" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A329" s="11"/>
-      <c r="B329" s="12"/>
-      <c r="C329" s="12"/>
-      <c r="D329" s="12"/>
-      <c r="E329" s="10"/>
-      <c r="F329" s="8"/>
-      <c r="G329" s="23"/>
-      <c r="H329" s="26"/>
-    </row>
-    <row r="330" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A330" s="11"/>
-      <c r="B330" s="12"/>
-      <c r="C330" s="12"/>
-      <c r="D330" s="12"/>
-      <c r="E330" s="10"/>
-      <c r="F330" s="8"/>
-      <c r="G330" s="23"/>
-      <c r="H330" s="26"/>
-    </row>
-    <row r="331" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A331" s="11"/>
-      <c r="B331" s="12"/>
-      <c r="C331" s="12"/>
-      <c r="D331" s="12"/>
-      <c r="E331" s="10"/>
-      <c r="F331" s="8"/>
-      <c r="G331" s="8"/>
-      <c r="H331" s="26"/>
-    </row>
-    <row r="332" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A332" s="11"/>
-      <c r="B332" s="12"/>
-      <c r="C332" s="12"/>
-      <c r="D332" s="12"/>
-      <c r="E332" s="10"/>
-      <c r="F332" s="8"/>
-      <c r="G332" s="23"/>
-      <c r="H332" s="26"/>
-    </row>
-    <row r="333" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A333" s="11"/>
-      <c r="B333" s="12"/>
-      <c r="C333" s="12"/>
-      <c r="D333" s="12"/>
-      <c r="E333" s="10"/>
-      <c r="F333" s="8"/>
-      <c r="G333" s="23"/>
-      <c r="H333" s="26"/>
-    </row>
-    <row r="334" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A334" s="11"/>
-      <c r="B334" s="12"/>
-      <c r="C334" s="12"/>
-      <c r="D334" s="12"/>
-      <c r="E334" s="10"/>
-      <c r="F334" s="8"/>
-      <c r="G334" s="23"/>
-      <c r="H334" s="26"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F124">

</xml_diff>